<commit_message>
docs: L2 report for the D13 session template unit
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CONDITIONING_TEMPLATES_V3_2026-07-25.xlsx
+++ b/docs/CONDITIONING_TEMPLATES_V3_2026-07-25.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A52"/>
+  <dimension ref="A1:A60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The Conditioning Templates — V3 (2026-07-25, Sam's rulings applied)</t>
+          <t>The Conditioning Templates — V3-FINAL (2026-07-25, all eight Sam rulings applied)</t>
         </is>
       </c>
     </row>
@@ -533,228 +533,232 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>SAM'S V3 RULINGS (2026-07-25) — all five applied</t>
+          <t>*** THE CLASSIFICATION LAW (Sam, V3-final) ***</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>1. SPRINT-FAMILY EXEMPTION from the 1:12 alactic ceiling: full recovery at 1:10–1:15+ is allowed. 9 ⚑ RATIO flags cleared (5 Acceleration, 4 Top End Speed).</t>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>INTENSITY CLASSIFIES. W:R IS ONLY A PROPERTY.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2. 150–200 m Hard Repeats: STRUCTURE changed to 'departing every 2:00' (not just relabelled). True ratio ~1:3–1:4, in band. Flag cleared.</t>
+          <t>A session belongs to the quality its INTENSITY says it belongs to. Its work-to-rest ratio describes the session; it does not decide which quality the session is. A W:R outside a quality's tabled band is therefore a property of that session, not a misfiling and not an error. Effort length reads the same way. This law governs every row in this sheet and retires the whole class of 'ratio outside band' flags: after it, 9 flags cleared at once (4 tempo rows, 3 protocol rows, and the two short-intermittent aerobic-power rows), leaving only genuinely INFERRED numbers to review.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>3. Extensive Tempo: session UNCHANGED, ratio label corrected to ~1:2 (the framework's '~2:1' was a labelling error).</t>
-        </is>
-      </c>
+      <c r="A9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>4. Repeated Jumps (5×3 broad jumps) DELETED entirely — jump work lives in the POWER SYSTEM only, not in conditioning. Bike power 8×6 s becomes 'Air Bike Accelerations' in the Acceleration tab. This resolves the V2 taxonomy flag as OPTION A: an alactic non-run variant lives in Acceleration via Modality Notes; no Anaerobic Power tab is added.</t>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>SAM'S RULINGS (2026-07-25) — all eight applied</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>5. FLUSH CONFIRMED at 7 rows: the 4 consolidated sessions (draft markers removed) plus 3 Sam-authored interval flushes (30:30, 1:1, 2:1), all at 3–4/10 MAX, any modality, mid-session mixing allowed.</t>
+          <t>1. SPRINT-FAMILY EXEMPTION from the 1:12 alactic ceiling: full recovery at 1:10–1:15+ is allowed. 9 ⚑ RATIO flags cleared (5 Acceleration, 4 Top End Speed).</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr"/>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2. 150–200 m Hard Repeats: STRUCTURE changed to 'departing every 2:00' (not just relabelled). True ratio ~1:3–1:4, in band. Flag cleared.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>THE GOVERNING TABLE (Sam's) — every row is checked against it</t>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>3. Extensive Tempo: session UNCHANGED, ratio label corrected to ~1:2 (the framework's '~2:1' was a labelling error).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Anaerobic power (alactic)          effort 3–10 s      W:R 1:6–1:12*     max speed and explosiveness</t>
+          <t>4. Repeated Jumps (5×3 broad jumps) DELETED entirely — jump work lives in the POWER SYSTEM only, not in conditioning. Bike power 8×6 s becomes 'Air Bike Accelerations' in the Acceleration tab. This resolves the V2 taxonomy flag as OPTION A: an alactic non-run variant lives in Acceleration via Modality Notes; no Anaerobic Power tab is added.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Repeated-sprint ability            effort 4–10 s      W:R 1:3–1:5       repeat high-speed efforts</t>
+          <t>5. FLUSH CONFIRMED at 7 rows: the 4 consolidated sessions (draft markers removed) plus 3 Sam-authored interval flushes (30:30, 1:1, 2:1), all at 3–4/10 MAX, any modality, mid-session mixing allowed.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Anaerobic capacity (glycolytic)    effort 15–60 s     W:R 1:2–1:5       sustain hard work through fatigue</t>
+          <t>6. V3-FINAL — INTENSITY CLASSIFIES, W:R IS ONLY A PROPERTY (the law above). The tempo cluster (30:30 controlled, 1 min on/1 min, 2 min on/1 min, extensive tempo) sits where its intensity says; all four flags cleared, along with every other ratio/effort-length flag on a non-inferred row.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Aerobic power                      effort 1–5 min     W:R 1:1–2:1       high aerobic output</t>
+          <t>7. V3-FINAL — 400 m Repeats depart every 3:00 (structure, not label): rest is the 3:00 remainder (≈100–105 s), ~1:1-ish aerobic power. Flag cleared.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Aerobic capacity                   longer/continuous     W:R 3:1–continuous    total sustainable aerobic work</t>
+          <t>8. V3-FINAL — Deceleration and Landing Work STAYS in Change of Direction-Decel: landing mechanics, not jump training (the deleted repeated-jumps session was jump training).</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>* SPRINT-FAMILY EXEMPTION (ruling 1): for alactic sprint work the 1:12 ceiling is NOT binding — full recovery at 1:10–1:15+ is allowed and is not flagged. The 1:6 floor still holds.</t>
-        </is>
-      </c>
+      <c r="A19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr"/>
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>THE GOVERNING TABLE (Sam's) — every row is checked against it</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>WHICH TAB MAPS TO WHICH FRAMEWORK QUALITY</t>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Anaerobic power (alactic)          effort 3–10 s      W:R 1:6–1:12*     max speed and explosiveness</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Acceleration + Top End Speed  -&gt;  anaerobic power (alactic). Acceleration now also holds the one non-run alactic row, Air Bike Accelerations (ruling 4).</t>
+          <t>Repeated-sprint ability            effort 4–10 s      W:R 1:3–1:5       repeat high-speed efforts</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Repeat Sprint                 -&gt;  repeated-sprint ability</t>
+          <t>Anaerobic capacity (glycolytic)    effort 15–60 s     W:R 1:2–1:5       sustain hard work through fatigue</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Anaerobic                     -&gt;  anaerobic capacity (glycolytic). GRIND IS DISSOLVED IN HERE (Sam's ruling).</t>
+          <t>Aerobic power                      effort 1–5 min     W:R 1:1–2:1       high aerobic output</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Aerobic Power                 -&gt;  aerobic power</t>
+          <t>Aerobic capacity                   longer/continuous     W:R 3:1–continuous    total sustainable aerobic work</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Aerobic Capacity              -&gt;  aerobic capacity</t>
+          <t>* SPRINT-FAMILY EXEMPTION (ruling 1): for alactic sprint work the 1:12 ceiling is NOT binding — full recovery at 1:10–1:15+ is allowed and is not flagged. The 1:6 floor still holds.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Change of Direction/Decel     -&gt;  NO framework row (mechanics quality) — unbanded, see Open Q6</t>
-        </is>
-      </c>
+      <c r="A27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Flush                         -&gt;  NO framework row (recovery, not a trained quality). 7 rows, confirmed.</t>
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>WHICH TAB MAPS TO WHICH FRAMEWORK QUALITY</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr"/>
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Acceleration + Top End Speed  -&gt;  anaerobic power (alactic). Acceleration now also holds the one non-run alactic row, Air Bike Accelerations (ruling 4).</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>THE SCHEMA (every row carries all six)</t>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Repeat Sprint                 -&gt;  repeated-sprint ability</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Work period — Rest period — Sets/rounds (reps) — Intensity (framework language: %MAS / %HRmax / effort words) — W:R ratio — Total session time. Total session time = work + rest only (add warm-up and cool-down on top).</t>
+          <t>Anaerobic                     -&gt;  anaerobic capacity (glycolytic). GRIND IS DISSOLVED IN HERE (Sam's ruling).</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr"/>
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Aerobic Power                 -&gt;  aerobic power</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>D14 — THE RENDERING LAYER FOR %MAS RUN WORK</t>
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Aerobic Capacity              -&gt;  aerobic capacity</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Every %MAS intensity in this sheet renders per-athlete through D14 (PROGRAMMING_DESIGN_SESSION_2026-07-23.md, 'MAS via 2 km time trial', Sam 2026-07-25): onboarding gains a 2 km TT screen (skippable — MAS then defaults by experience level so every MAS session still renders); MAS is stored on-device; %MAS intensities become per-athlete paces and rep distances; a 2 km TT is re-prescribed as a real aerobic-power session every ~6–8 weeks to recalibrate. So '90–100% MAS' in these rows is a rendering instruction, not a fixed pace.</t>
+          <t>Change of Direction/Decel     -&gt;  NO framework row (mechanics quality) — unbanded, see Open Q6</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr"/>
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Flush                         -&gt;  NO framework row (recovery, not a trained quality). 7 rows, confirmed.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="3" t="inlineStr">
-        <is>
-          <t>THE ⚑ FLAGS</t>
-        </is>
-      </c>
+      <c r="A36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>⚑ RATIO — computed W:R outside the quality's band (band shown). ⚑ BAND — effort length or intensity outside the quality's column, ratio fine. ⚑ INFERRED — the numbers are this sheet's invention, not a citation. Flagged rows are SHADED and listed on the 'Skim List' tab. Nothing is silently re-dosed — every fix is Sam's call.</t>
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>THE SCHEMA (every row carries all six)</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr"/>
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Work period — Rest period — Sets/rounds (reps) — Intensity (framework language: %MAS / %HRmax / effort words) — W:R ratio — Total session time. Total session time = work + rest only (add warm-up and cool-down on top).</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>EFFORT-LENGTH ASSUMPTIONS (used to compute work periods and W:R from distance rows)</t>
-        </is>
-      </c>
+      <c r="A39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>10 m ≈ 2 s  ·  20 m ≈ 3 s  ·  20 m shuttle (2×10 m) ≈ 4 s  ·  30 m ≈ 4.5 s  ·  40–60 m ≈ 6–8 s  ·  20+20 fly ≈ 6 s  ·  30+30 fly ≈ 8 s</t>
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>D14 — THE RENDERING LAYER FOR %MAS RUN WORK</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>100 m @65–75% ≈ 16 s  ·  150 m ≈ 22 s  ·  200 m ≈ 30 s  ·  400 m ≈ 75–80 s  ·  1 km ≈ 3.5–4 min. Walk-back/walk-down recovery is timed, not assumed instant.</t>
+          <t>Every %MAS intensity in this sheet renders per-athlete through D14 (PROGRAMMING_DESIGN_SESSION_2026-07-23.md, 'MAS via 2 km time trial', Sam 2026-07-25): onboarding gains a 2 km TT screen (skippable — MAS then defaults by experience level so every MAS session still renders); MAS is stored on-device; %MAS intensities become per-athlete paces and rep distances; a 2 km TT is re-prescribed as a real aerobic-power session every ~6–8 weeks to recalibrate. So '90–100% MAS' in these rows is a rendering instruction, not a fixed pace.</t>
         </is>
       </c>
     </row>
@@ -764,64 +768,112 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>STANDING RENDERING RULES</t>
+          <t>THE ⚑ FLAGS</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>1. TIME-FIRST. Distance is allowed for short/speed work and mid-length reps; calories for EMOM-class erg work.</t>
+          <t>After the classification law, ⚑ RATIO and ⚑ BAND are retired as a class: a ratio or effort length outside a tabled band is a property, not a fault. ONE ratio mark survives, on an optional variant Sam has not ruled on (the descending-rest option inside 45 s Hard Repeats). Everything else still marked is ⚑ INFERRED — the numbers are this sheet's invention, not a citation. Flagged rows are SHADED and listed on the 'Skim List' tab, which is now the whole review queue.</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>2. Run/Ski/Row share the nominal distance. Bike = distance × 2. Air Bike is time-based: 250 m ≈ 1 min.</t>
-        </is>
-      </c>
+      <c r="A45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>3. Work intervals over 8 min: Run and Bike only. Ski/Row/Air Bike cap at 8 min, prefer 6. Encoded per row.</t>
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>EFFORT-LENGTH ASSUMPTIONS (used to compute work periods and W:R from distance rows)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>4. Sprint-family templates are run-only, with THREE named exceptions encoded in Modality Notes: AIR BIKE ACCELERATIONS (ruling 4 — an alactic air-bike row inside Acceleration); the 30 m repeats' Air-Bike-extra rendering (5 s effort / 30 s super-light); and anything under 10 s of sprinting staying on running or the Air Bike.</t>
+          <t>10 m ≈ 2 s  ·  20 m ≈ 3 s  ·  20 m shuttle (2×10 m) ≈ 4 s  ·  30 m ≈ 4.5 s  ·  40–60 m ≈ 6–8 s  ·  20+20 fly ≈ 6 s  ·  30+30 fly ≈ 8 s</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>5. NO SLEDS anywhere. GRIND folded into ANAEROBIC. Jump work lives in the POWER SYSTEM only (ruling 4).</t>
+          <t>100 m @65–75% ≈ 16 s  ·  150 m ≈ 22 s  ·  200 m ≈ 30 s  ·  400 m ≈ 75–80 s  ·  1 km ≈ 3.5–4 min. Walk-back/walk-down recovery is timed, not assumed instant.</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>6. MID-SESSION MIXING — FLUSH-ONLY PROPERTY (ruling 5). On the three Flush Intervals rows the athlete may rotate machines and/or running BETWEEN ROUNDS within one session. This is the only place in the sheet where a single session spans modalities; everywhere else one session renders on one modality.</t>
-        </is>
-      </c>
+      <c r="A49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr"/>
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>STANDING RENDERING RULES</t>
+        </is>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t>HOW TO READ THE CHANGE MARKS</t>
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>1. TIME-FIRST. Distance is allowed for short/speed work and mid-length reps; calories for EMOM-class erg work.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>2. Run/Ski/Row share the nominal distance. Bike = distance × 2. Air Bike is time-based: 250 m ≈ 1 min.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>3. Work intervals over 8 min: Run and Bike only. Ski/Row/Air Bike cap at 8 min, prefer 6. Encoded per row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>4. Sprint-family templates are run-only, with THREE named exceptions encoded in Modality Notes: AIR BIKE ACCELERATIONS (ruling 4 — an alactic air-bike row inside Acceleration); the 30 m repeats' Air-Bike-extra rendering (5 s effort / 30 s super-light); and anything under 10 s of sprinting staying on running or the Air Bike.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>5. NO SLEDS anywhere. GRIND folded into ANAEROBIC. Jump work lives in the POWER SYSTEM only (ruling 4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>6. MID-SESSION MIXING — FLUSH-ONLY PROPERTY (ruling 5). On the three Flush Intervals rows the athlete may rotate machines and/or running BETWEEN ROUNDS within one session. This is the only place in the sheet where a single session spans modalities; everywhere else one session renders on one modality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>7. INTENSITY CLASSIFIES, W:R IS ONLY A PROPERTY (Sam, V3-final) — see the law at the top of this tab. Do not re-file a session because its ratio sits outside a band, and do not re-dose it to fit one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>HOW TO READ THE CHANGE MARKS</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>MOVED = re-filed to a different quality tab. MERGED = one or more templates folded in (named). SPLIT = one template became two rows. FRAMEWORK-ALIGNED = dose replaced by the framework's numbers. SCHEMA-FILLED = a missing work/rest/set value supplied. NEW = added by a V3 ruling. CONFIRMED = a V2 draft Sam has now signed off. The Change Log tab traces all 99 V2-base rows plus the V3 additions.</t>
         </is>
@@ -5041,7 +5093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5185,218 +5237,262 @@
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>R6</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>STILL OPEN — the tempo family sits outside the aerobic-capacity band  [BIGGEST REMAINING FLAG CLUSTER]</t>
+          <t>RESOLVED — the tempo-family band question (was the biggest open cluster)</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>30:30 controlled (1:1), 1 min on/1 min easy (1:1), 2 min on/1 min easy (2:1) and extensive tempo (≈1:2) run at capacity INTENSITY but at aerobic-power RATIOS. The 3:1–continuous band has no room for them. 4 of the 6 non-inferred ⚑ RATIO marks left in the sheet are these rows. NOTE: your V3 ruling 3 answered the extensive-tempo LABEL, which was a different question from this one.</t>
+          <t>Sam's law: INTENSITY CLASSIFIES, W:R IS ONLY A PROPERTY. The tempo cluster sits where its intensity says.</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>Add a Tempo/threshold quality; or widen the aerobic-capacity band to admit intensity-defined tempo intervals; or accept the four rows as permanently flagged. Your ruling-5 flush rows show the principle that would settle it: there, an INTENSITY CAP (3–4/10) is what decides the quality, not the ratio.</t>
+          <t>Applied. 30:30 controlled, 1 min on/1 min, 2 min on/1 min and extensive tempo all cleared and stay in Aerobic Capacity. The same law retired every other ratio/effort-length flag on a non-inferred row.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>Q4b</t>
+          <t>R7</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>STILL OPEN — 400 m Repeats at 1:1.6</t>
+          <t>RESOLVED — 400 m Repeats at 1:1.6</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>The one remaining non-inferred, non-tempo ⚑ RATIO row: 400 m (≈75–80 s) with 2 min rest is 1:1.6, outside the aerobic-power band 1:1–2:1 (which requires rest &lt;= work).</t>
+          <t>Sam: departing every 3:00 (structure, not label).</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>The ruling-2 move would work here too: 'departing every 2:30' gives ≈1:1 and clears it. Or confirm 1:1.6 and widen the band. Related: the 60–90 s row's 90 s effort still exceeds the 15–60 s column.</t>
+          <t>Applied. Rest is the 3:00 remainder (≈100–105 s); ≈1:1.3, and exactly 1:1 for an athlete running ≈90 s. Flag cleared.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Q6</t>
+          <t>R8</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>STILL OPEN — COD/Decel is not a row in the governing table</t>
+          <t>RESOLVED — Q14, the landing row</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>6 rows, unbanded; 5 of them still ⚑ INFERRED.</t>
+          <t>Sam: Deceleration and Landing Work stays in COD — landing mechanics, not jump training.</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>Keep as an explicitly unbanded mechanics tab; or fold into anaerobic power / RSA; or author a COD line in the framework.</t>
+          <t>Applied. The row keeps only its ⚑ INFERRED dose mark.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>Q14</t>
+          <t>R12</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>NEW — does 'jump work is power-system only' reach the COD landing row?</t>
+          <t>RESOLVED (by the law) — 30 m Acceleration Reps intensity</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Ruling 4 deleted the repeated-jumps session. ⚑ 'Deceleration and Landing Work' (jump-land-stick / run-and-stick) is still in Change of Direction-Decel. It reads as landing MECHANICS rather than jump training, so it was left in place rather than deleted by inference.</t>
+          <t>The '80–90%' in your cue is a top-end-VELOCITY instruction, not a metabolic intensity, so the row classifies as maximal-intent alactic acceleration.</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Confirm it stays as decel mechanics, or delete it too and let the power system own all landing work.</t>
+          <t>Flag cleared on that reading. If you meant 80–90% metabolically, say so and it comes back.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>Q9</t>
+          <t>Q6</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>STILL OPEN — Off-Feet MetCon removed in both places</t>
+          <t>STILL OPEN — COD/Decel is not a row in the governing table</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>You marked the Grind copy 'remove for now'; the Aerobic Power copy was the same template cross-listed, so it left with it.</t>
+          <t>6 rows, unbanded; 5 of them still ⚑ INFERRED.</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>Confirm — or say the word and the VO2-reading copy returns with a concrete work/rest structure.</t>
+          <t>Keep as an explicitly unbanded mechanics tab; or fold into anaerobic power / RSA; or author a COD line in the framework.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>Q10</t>
+          <t>Q14</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>STILL OPEN — the 10 s boundary on Row/Ski</t>
+          <t>NEW — does 'jump work is power-system only' reach the COD landing row?</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Your rule reads 'anything under 10 seconds of sprinting keep to running or air bike'. The 10 s Max Sprint Repeats row sits exactly on the boundary, so Row/Ski are currently excluded from it.</t>
+          <t>Ruling 4 deleted the repeated-jumps session. ⚑ 'Deceleration and Landing Work' (jump-land-stick / run-and-stick) is still in Change of Direction-Decel. It reads as landing MECHANICS rather than jump training, so it was left in place rather than deleted by inference.</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Confirm 10 s counts as 'under 10 s', or allow Row/Ski at exactly 10 s.</t>
+          <t>Confirm it stays as decel mechanics, or delete it too and let the power system own all landing work.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Q12</t>
+          <t>Q9</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>STILL OPEN — 30 m Acceleration Reps intensity</t>
+          <t>STILL OPEN — Off-Feet MetCon removed in both places</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Its cue caps the rep at 80–90%; the framework's alactic intensity is 95–100%. (⚑ BAND, not RATIO.)</t>
+          <t>You marked the Grind copy 'remove for now'; the Aerobic Power copy was the same template cross-listed, so it left with it.</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>Confirm the cue governs, or raise the row to 95–100%.</t>
+          <t>Confirm — or say the word and the VO2-reading copy returns with a concrete work/rest structure.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>Q13</t>
+          <t>Q10</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>STILL OPEN — ⚑ Resisted Band Acceleration</t>
+          <t>STILL OPEN — the 10 s boundary on Row/Ski</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>In neither the Bible nor the framework; its numbers are this sheet's invention. It is a band, not a sled.</t>
+          <t>Your rule reads 'anything under 10 seconds of sprinting keep to running or air bike'. The 10 s Max Sprint Repeats row sits exactly on the boundary, so Row/Ski are currently excluded from it.</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Keep as an ⚑ INFERRED option, or remove it the way the sled row went.</t>
+          <t>Confirm 10 s counts as 'under 10 s', or allow Row/Ski at exactly 10 s.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>Q8</t>
+          <t>Q12</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>ANSWERED BY IMPLICATION — Air Bike in Flush</t>
+          <t>STILL OPEN — 30 m Acceleration Reps intensity</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Ruling 5 makes the three new flushes ANY-modality with mixing, which admits the Air Bike to Flush. The Bible's L501 caveat was about air-bike SPRINTS called recovery, not an easy spin.</t>
+          <t>Its cue caps the rep at 80–90%; the framework's alactic intensity is 95–100%. (⚑ BAND, not RATIO.)</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>No action taken beyond allowing it. Say so if you want Air Bike struck from Flush explicitly.</t>
+          <t>Confirm the cue governs, or raise the row to 95–100%.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
+          <t>Q13</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>STILL OPEN — ⚑ Resisted Band Acceleration</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>In neither the Bible nor the framework; its numbers are this sheet's invention. It is a band, not a sled.</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Keep as an ⚑ INFERRED option, or remove it the way the sled row went.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Q8</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>ANSWERED BY IMPLICATION — Air Bike in Flush</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Ruling 5 makes the three new flushes ANY-modality with mixing, which admits the Air Bike to Flush. The Bible's L501 caveat was about air-bike SPRINTS called recovery, not an easy spin.</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>No action taken beyond allowing it. Say so if you want Air Bike struck from Flush explicitly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
           <t>Q11</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>PARTLY RESOLVED — framework sessions with no template row</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>Repeated jumps: DELETED by ruling 4. Bike power: now Air Bike Accelerations. THREE remain untemplated.</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>Still with no row (say the word and they are built): 30:15 intervals (2×10 reps 30s/15s float, 3 min between — aerobic power); hard shuttles 2×4×30 s (90 s rest, 4 min between — anaerobic); footy repeat efforts 3×4×20 s shuttle (60 s rest, 3 min between — anaerobic).</t>
         </is>
@@ -5413,7 +5509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5464,39 +5560,39 @@
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>30 m Acceleration Reps</t>
+          <t>⚑ Resisted Band Acceleration</t>
         </is>
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>BAND</t>
+          <t>INFERRED</t>
         </is>
       </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
-          <t>1:27 (approx)</t>
+          <t>1:30 (approx)</t>
         </is>
       </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
-          <t>Open Q12 - intensity 80-90% vs the alactic 95-100%</t>
+          <t>Open Q13 - keep as an INFERRED option or remove it the way the sled row went</t>
         </is>
       </c>
       <c r="F2" s="8" t="inlineStr">
         <is>
-          <t>⚑ BAND: intensity 80–90% sits below the framework's 95–100% alactic intensity — Sam's cue governs; confirm (Open Q12). Ratio exempt per ruling 1.</t>
+          <t>IN BAND — SPRINT-FAMILY EXEMPTION (Sam's V3 ruling 1): full recovery at 1:10–1:15+ is allowed above the table's 1:12 ceiling for alactic sprint work. ⚑ INFERRED numbers.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>Acceleration</t>
+          <t>Repeat Sprint</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>⚑ Resisted Band Acceleration</t>
+          <t>⚑ Inverse Tabata</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
@@ -5506,49 +5602,49 @@
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
-          <t>1:30 (approx)</t>
+          <t>1:2</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>Open Q13 - keep as INFERRED or remove</t>
+          <t>Numbers are the sheet's invention - confirm the dose or replace it</t>
         </is>
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>IN BAND — SPRINT-FAMILY EXEMPTION (Sam's V3 ruling 1): full recovery at 1:10–1:15+ is allowed above the table's 1:12 ceiling for alactic sprint work. ⚑ INFERRED numbers.</t>
+          <t>IN BAND. CLASSIFIED BY INTENSITY (Sam's V3-final law: intensity classifies, W:R is only a property). A 10 s maximal effort classifies as repeat-sprint work; the 1:2 W:R is a property (10 s / 30 s would also read 1:3 if you prefer it). ⚑ INFERRED timing — the only mark left on this row.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>Repeat Sprint</t>
+          <t>Change of Direction-Decel</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>⚑ Inverse Tabata</t>
+          <t>⚑ Low-Intensity Deceleration Drills</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>RATIO + INFERRED</t>
+          <t>INFERRED</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>1:2</t>
+          <t>≈1:8</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>Confirm the dose (INFERRED) and the ratio together, or bin the row</t>
+          <t>Dose is INFERRED (the Bible names the drill, not the numbers). Confirm the numbers or replace them. Q6 (COD has no framework band) is still open.</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>⚑ RATIO 1:2 vs band 1:3–1:5 — 10 s / 30 s would put it in band (Sam's one-line call). ⚑ INFERRED timing.</t>
+          <t>No framework band — COD/Decel is not a row in Sam's governing table (mechanics quality). W:R shown for information only. See Open Q6. ⚑ INFERRED numbers.</t>
         </is>
       </c>
     </row>
@@ -5560,7 +5656,7 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>⚑ Low-Intensity Deceleration Drills</t>
+          <t>⚑ Deceleration and Landing Work</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
@@ -5570,17 +5666,17 @@
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>≈1:8</t>
+          <t>≈1:12</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>Open Q6 (no framework band) / Q14 for the landing row - dose is INFERRED</t>
+          <t>Dose is INFERRED (the Bible names the drill, not the numbers). Confirm the numbers or replace them. Q6 (COD has no framework band) is still open.</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>No framework band — COD/Decel is not a row in Sam's governing table (mechanics quality). W:R shown for information only. See Open Q6. ⚑ INFERRED numbers.</t>
+          <t>No framework band — COD/Decel is not a row in Sam's governing table (mechanics quality). W:R shown for information only. See Open Q6. STAYS IN COD per Sam's V3-final ruling 3: landing MECHANICS, not jump training (the deleted repeated-jumps session was jump training). ⚑ INFERRED numbers — the only mark left on this row.</t>
         </is>
       </c>
     </row>
@@ -5592,7 +5688,7 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>⚑ Deceleration and Landing Work</t>
+          <t>⚑ Short COD Circuit</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
@@ -5602,12 +5698,12 @@
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>≈1:12</t>
+          <t>≈1:7</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Open Q6 (no framework band) / Q14 for the landing row - dose is INFERRED</t>
+          <t>Dose is INFERRED (the Bible names the drill, not the numbers). Confirm the numbers or replace them. Q6 (COD has no framework band) is still open.</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
@@ -5624,7 +5720,7 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>⚑ Short COD Circuit</t>
+          <t>⚑ 45-Degree Cut Reps</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
@@ -5634,12 +5730,12 @@
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>≈1:7</t>
+          <t>≈1:20</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>Open Q6 (no framework band) / Q14 for the landing row - dose is INFERRED</t>
+          <t>Dose is INFERRED (the Bible names the drill, not the numbers). Confirm the numbers or replace them. Q6 (COD has no framework band) is still open.</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
@@ -5656,7 +5752,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>⚑ 45-Degree Cut Reps</t>
+          <t>⚑ COD Finisher (occasional, off-season only)</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -5666,29 +5762,29 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>≈1:20</t>
+          <t>≈1:3</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Open Q6 (no framework band) / Q14 for the landing row - dose is INFERRED</t>
+          <t>Dose is INFERRED (the Bible names the drill, not the numbers). Confirm the numbers or replace them. Q6 (COD has no framework band) is still open.</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>No framework band — COD/Decel is not a row in Sam's governing table (mechanics quality). W:R shown for information only. See Open Q6. ⚑ INFERRED numbers.</t>
+          <t>No framework band — COD/Decel is not a row in Sam's governing table (mechanics quality). W:R shown for information only. See Open Q6. ⚑ INFERRED dose.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Change of Direction-Decel</t>
+          <t>Anaerobic</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>⚑ COD Finisher (occasional, off-season only)</t>
+          <t>⚑ Tabata Intervals</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
@@ -5698,17 +5794,17 @@
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>≈1:3</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>Open Q6 (no framework band) / Q14 for the landing row - dose is INFERRED</t>
+          <t>Numbers are the sheet's invention - confirm the dose or replace it</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>No framework band — COD/Decel is not a row in Sam's governing table (mechanics quality). W:R shown for information only. See Open Q6. ⚑ INFERRED dose.</t>
+          <t>IN BAND. CLASSIFIED BY INTENSITY (Sam's V3-final law: intensity classifies, W:R is only a property). Supramaximal glycolytic intensity classifies it in Anaerobic; the work-heavy 2:1 is a property of the protocol. ⚑ INFERRED timing — the only mark left on this row.</t>
         </is>
       </c>
     </row>
@@ -5720,27 +5816,27 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>⚑ Tabata Intervals</t>
+          <t>45 s Hard Repeats</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>RATIO + INFERRED</t>
+          <t>RATIO</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>1:2.7</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>Confirm the dose (INFERRED) and the ratio together, or bin the row</t>
+          <t>VARIANT ONLY - the base row is in band and unflagged. Confirm or drop the descending-rest option (1:0.7 at the last rep). The one ratio mark left in the sheet.</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>⚑ RATIO 2:1 vs band 1:2–1:5 (work-heavy by a wide margin). ⚑ INFERRED timing.</t>
+          <t>IN BAND (15–60 s, 1:2–1:5). Descending-rest variant (90 s —&gt; 30 s across reps) carries ⚑ RATIO 1:0.7 at the last rep vs band 1:2–1:5.</t>
         </is>
       </c>
     </row>
@@ -5752,347 +5848,59 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>45 s Hard Repeats</t>
+          <t>⚑ Bodyweight Grind Circuit (no-equipment fallback)</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>RATIO</t>
+          <t>INFERRED</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>1:2.7</t>
+          <t>≈2:1</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>VARIANT ONLY - the base row is in band. Confirm or drop the descending-rest option (1:0.7 at the last rep).</t>
+          <t>Numbers are the sheet's invention - confirm the dose or replace it</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>IN BAND (15–60 s, 1:2–1:5). Descending-rest variant (90 s —&gt; 30 s across reps) carries ⚑ RATIO 1:0.7 at the last rep vs band 1:2–1:5.</t>
+          <t>IN BAND. CLASSIFIED BY INTENSITY (Sam's V3-final law: intensity classifies, W:R is only a property). Sustained hard circuit intensity classifies it in Anaerobic; the work-heavy ratio is a property of the circuit format. ⚑ INFERRED numbers — the only mark left on this row.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>Anaerobic</t>
+          <t>Aerobic Power</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>60–90 s Max Sustained Effort</t>
+          <t>⚑ Erg EMOM</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>BAND</t>
+          <t>INFERRED</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>1:2 (Sam)</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>Open Q4b - confirm the 90 s effort stays above the 15-60 s column</t>
+          <t>Numbers are the sheet's invention - confirm the dose or replace it</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>⚑ BAND: 90 s effort is above the framework's 15–60 s ceiling (Sam's own row + his 1:2 ruling) — confirm 90 s stays (Open Q4b). W:R in band.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>Anaerobic</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>⚑ Bodyweight Grind Circuit (no-equipment fallback)</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>RATIO + INFERRED</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>≈2:1</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>Confirm the dose (INFERRED) and the ratio together, or bin the row</t>
-        </is>
-      </c>
-      <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>⚑ RATIO ≈2:1 vs band 1:2–1:5 (circuit format is work-heavy). ⚑ INFERRED numbers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>Aerobic Power</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>MAS 15:15 Blocks</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>BAND</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>1:1</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>Effort-length note only - confirm the framework's own 30:15 session is the precedent for short intermittent work in Aerobic Power.</t>
-        </is>
-      </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>W:R IN BAND. ⚑ BAND: 15 s effort is below the 1–5 min column — the framework's own 30:15 session sets the short-intermittent precedent.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>Aerobic Power</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>30:30 Hard Intermittent</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>BAND</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>1:1</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>Effort-length note only - confirm the framework's own 30:15 session is the precedent for short intermittent work in Aerobic Power.</t>
-        </is>
-      </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>W:R IN BAND. ⚑ BAND: 30 s effort below the 1–5 min column (same 30:15 precedent as above).</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>Aerobic Power</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>400 m Repeats</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>RATIO</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>1:1.6</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>Open Q4b - 'departing every 2:30' would clear it the way ruling 2 did</t>
-        </is>
-      </c>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>⚑ RATIO 1:1.6 vs band 1:1–2:1 (rest exceeds work). Rest ≈75–80 s would put it in band — Sam's call, not silently changed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>Aerobic Power</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>⚑ Erg EMOM</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>BAND + INFERRED</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>Confirm the INFERRED split, plus the same short-intermittent effort-length note as MAS 15:15 / 30:30.</t>
-        </is>
-      </c>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>W:R IN BAND. ⚑ BAND: 40 s effort below the 1–5 min column (30:15 precedent). ⚑ INFERRED per-minute split.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
-        <is>
-          <t>Aerobic Capacity</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>Extensive Tempo (100 m repeats)</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>RATIO</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>≈1:2</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="inlineStr">
-        <is>
-          <t>Open Q3 (tempo band) - the biggest remaining cluster</t>
-        </is>
-      </c>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>⚑ RATIO ≈1:2 vs band 3:1–continuous — the whole tempo-interval family (30:30, 1:1, 2:1) sits outside the aerobic-capacity band. One systemic question, see Open Q3. LABEL CORRECTED to ~1:2 by Sam's V3 ruling 3 (the framework's '~2:1' was a labelling error) — the SESSION IS UNCHANGED. The surviving flag is the band question in Open Q3, not the label.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="8" t="inlineStr">
-        <is>
-          <t>Aerobic Capacity</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>2 min On / 1 min Easy</t>
-        </is>
-      </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>RATIO</t>
-        </is>
-      </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="inlineStr">
-        <is>
-          <t>Open Q3 (tempo band) - the biggest remaining cluster</t>
-        </is>
-      </c>
-      <c r="F19" s="8" t="inlineStr">
-        <is>
-          <t>⚑ RATIO 2:1 vs band 3:1–continuous — the whole tempo-interval family (30:30, 1:1, 2:1) sits outside the aerobic-capacity band. One systemic question, see Open Q3.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
-        <is>
-          <t>Aerobic Capacity</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>30:30 Controlled Tempo Blocks</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>RATIO</t>
-        </is>
-      </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>1:1</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>Open Q3 (tempo band) - the biggest remaining cluster</t>
-        </is>
-      </c>
-      <c r="F20" s="8" t="inlineStr">
-        <is>
-          <t>⚑ RATIO 1:1 vs band 3:1–continuous — the whole tempo-interval family (30:30, 1:1, 2:1) sits outside the aerobic-capacity band. One systemic question, see Open Q3.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t>Aerobic Capacity</t>
-        </is>
-      </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>1 min On / 1 min Easy Tempo</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>RATIO</t>
-        </is>
-      </c>
-      <c r="D21" s="8" t="inlineStr">
-        <is>
-          <t>1:1</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="inlineStr">
-        <is>
-          <t>Open Q3 (tempo band) - the biggest remaining cluster</t>
-        </is>
-      </c>
-      <c r="F21" s="8" t="inlineStr">
-        <is>
-          <t>⚑ RATIO 1:1 vs band 3:1–continuous — the whole tempo-interval family (30:30, 1:1, 2:1) sits outside the aerobic-capacity band. One systemic question, see Open Q3.</t>
+          <t>IN BAND. CLASSIFIED BY INTENSITY (Sam's V3-final law: intensity classifies, W:R is only a property). Hard aerobic intensity classifies it here; the 40 s effort length is a property (30:15 precedent). ⚑ INFERRED per-minute split — the only mark left on this row.</t>
         </is>
       </c>
     </row>
@@ -6107,7 +5915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6251,20 +6059,86 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>INTENSITY CLASSIFIES, W:R IS ONLY A PROPERTY (new law in the framework + Architecture tab)</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>9 flags cleared on non-inferred rows: the 4 tempo rows (30:30 controlled, 1 min on/1 min, 2 min on/1 min, extensive tempo), MAS 15:15 and 30:30 Hard Intermittent (short-intermittent effort length), 60-90 s Max Sustained (90 s effort), 30 m Acceleration Reps (velocity cue read as velocity, not metabolic intensity), and the ratio marks on 3 INFERRED protocol rows (Tabata, Inverse Tabata, Bodyweight Circuit), which stay flagged as INFERRED only</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>APPLIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>400 m Repeats: departing every 3:00 (structure, not label)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>1 row - rest is now the 3:00 remainder (≈100-105 s); ~1:1.3, or 1:1 for an athlete running ≈90 s; flag cleared</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>APPLIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Deceleration and Landing Work stays in COD - landing mechanics, not jump training</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>1 row - Q14 closed; the row keeps only its ⚑ INFERRED dose mark</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>APPLIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
           <t>D14</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Note the 2 km TT -&gt; MAS personalisation as the rendering layer for %MAS run work</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>Recorded on the Architecture tab, citing PROGRAMMING_DESIGN_SESSION_2026-07-23.md D14 (2 km TT screen, skippable with experience-level defaults, on-device MAS, ~6-8 week re-test)</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>RECORDED</t>
         </is>
@@ -6300,17 +6174,17 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>v2 rows</t>
+          <t>V3-final rows</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>⚑ RATIO</t>
+          <t>⚑ RATIO (retired as a class)</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>⚑ BAND</t>
+          <t>⚑ BAND (retired)</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
@@ -6337,7 +6211,7 @@
         <v>0</v>
       </c>
       <c r="D2" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2" s="5" t="n">
         <v>1</v>
@@ -6378,7 +6252,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4" s="5" t="n">
         <v>0</v>
@@ -6422,10 +6296,10 @@
         <v>9</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>2</v>
@@ -6444,10 +6318,10 @@
         <v>9</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E7" s="5" t="n">
         <v>1</v>
@@ -6466,7 +6340,7 @@
         <v>10</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D8" s="5" t="n">
         <v>0</v>
@@ -6510,10 +6384,10 @@
         <v>58</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E10" s="6" t="n">
         <v>10</v>
@@ -6801,67 +6675,67 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>30 m Acceleration Reps</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>kept</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>≈4.5 s (30 m)</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>2 min (full recovery)</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>4–6 reps</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>~80–90% build, no top-end (Sam's own cue caps it)</t>
         </is>
       </c>
-      <c r="G4" s="8" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>1:27 (approx)</t>
         </is>
       </c>
-      <c r="H4" s="8" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>≈11 min (work ≈27 s)</t>
         </is>
       </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>⚑ BAND: intensity 80–90% sits below the framework's 95–100% alactic intensity — Sam's cue governs; confirm (Open Q12). Ratio exempt per ruling 1.</t>
-        </is>
-      </c>
-      <c r="J4" s="8" t="inlineStr">
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>IN BAND. CLASSIFIED BY INTENSITY (Sam's V3-final law: intensity classifies, W:R is only a property). The '80–90%' in the cue is a TOP-END-VELOCITY instruction (no top-end on a 30 m rep), not a metabolic intensity — the effort is still maximal-intent alactic acceleration, so the row classifies here. Ratio exempt per ruling 1. (If you meant 80–90% metabolically, say so and the flag returns.)</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>Longer accel, still no top-end — build to about 80–90% and hold form.</t>
         </is>
       </c>
-      <c r="K4" s="8" t="inlineStr">
+      <c r="K4" s="5" t="inlineStr">
         <is>
           <t>distance (30 m ≈ 4.5 s)</t>
         </is>
       </c>
-      <c r="L4" s="8" t="inlineStr">
+      <c r="L4" s="5" t="inlineStr">
         <is>
           <t>Run-only (field sprint/cutting mechanics; rule 4). No machine rendering.</t>
         </is>
       </c>
-      <c r="M4" s="8" t="inlineStr">
+      <c r="M4" s="5" t="inlineStr">
         <is>
           <t>Bible Sect.7 Acceleration L1549; rest + W:R + total computed in v2</t>
         </is>
@@ -7973,7 +7847,7 @@
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
-          <t>⚑ RATIO 1:2 vs band 1:3–1:5 — 10 s / 30 s would put it in band (Sam's one-line call). ⚑ INFERRED timing.</t>
+          <t>IN BAND. CLASSIFIED BY INTENSITY (Sam's V3-final law: intensity classifies, W:R is only a property). A 10 s maximal effort classifies as repeat-sprint work; the 1:2 W:R is a property (10 s / 30 s would also read 1:3 if you prefer it). ⚑ INFERRED timing — the only mark left on this row.</t>
         </is>
       </c>
       <c r="J6" s="8" t="inlineStr">
@@ -8270,7 +8144,7 @@
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
-          <t>No framework band — COD/Decel is not a row in Sam's governing table (mechanics quality). W:R shown for information only. See Open Q6. ⚑ INFERRED numbers.</t>
+          <t>No framework band — COD/Decel is not a row in Sam's governing table (mechanics quality). W:R shown for information only. See Open Q6. STAYS IN COD per Sam's V3-final ruling 3: landing MECHANICS, not jump training (the deleted repeated-jumps session was jump training). ⚑ INFERRED numbers — the only mark left on this row.</t>
         </is>
       </c>
       <c r="J4" s="8" t="inlineStr">
@@ -8768,7 +8642,7 @@
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
-          <t>⚑ RATIO 2:1 vs band 1:2–1:5 (work-heavy by a wide margin). ⚑ INFERRED timing.</t>
+          <t>IN BAND. CLASSIFIED BY INTENSITY (Sam's V3-final law: intensity classifies, W:R is only a property). Supramaximal glycolytic intensity classifies it in Anaerobic; the work-heavy 2:1 is a property of the protocol. ⚑ INFERRED timing — the only mark left on this row.</t>
         </is>
       </c>
       <c r="J4" s="8" t="inlineStr">
@@ -8927,67 +8801,67 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>60–90 s Max Sustained Effort</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>MOVED (GRIND DISSOLVED) + MERGED — folds in ⚑ '1-Minute Effort Ladder'. Rest set by SAM'S OWN EDIT: 1:2 work-to-rest.</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>60–90 s all-out</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>2–3 min (Sam's 1:2 ruling)</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>4–6 reps</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>All-out sustained — unpleasant by 45 s</t>
         </is>
       </c>
-      <c r="G7" s="8" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>1:2 (Sam)</t>
         </is>
       </c>
-      <c r="H7" s="8" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>≈14–21 min (hard work 4–9 min)</t>
         </is>
       </c>
-      <c r="I7" s="8" t="inlineStr">
-        <is>
-          <t>⚑ BAND: 90 s effort is above the framework's 15–60 s ceiling (Sam's own row + his 1:2 ruling) — confirm 90 s stays (Open Q4b). W:R in band.</t>
-        </is>
-      </c>
-      <c r="J7" s="8" t="inlineStr">
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>IN BAND. CLASSIFIED BY INTENSITY (Sam's V3-final law: intensity classifies, W:R is only a property). All-out sustained effort is glycolytic intensity, so the row classifies in Anaerobic; the 90 s upper end sitting above the 15–60 s column is a property, not a misfiling. W:R 1:2 per Sam.</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>This is the zone the Bible means by 'grind for up to 1 min' — it should feel unpleasant by 45 seconds in.</t>
         </is>
       </c>
-      <c r="K7" s="8" t="inlineStr">
+      <c r="K7" s="5" t="inlineStr">
         <is>
           <t>time</t>
         </is>
       </c>
-      <c r="L7" s="8" t="inlineStr">
+      <c r="L7" s="5" t="inlineStr">
         <is>
           <t>All 5 modalities (time-based). Run: the 150–200 m repeats below are the running-native equivalent.</t>
         </is>
       </c>
-      <c r="M7" s="8" t="inlineStr">
+      <c r="M7" s="5" t="inlineStr">
         <is>
           <t>Bible L1483 ('grind for up to 1 min') + Sam's edit '1:2 work to rest ratio'</t>
         </is>
@@ -9001,7 +8875,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>SPLIT from Aerobic Power's '200m/400m Repeats' (200 m ≈30 s is glycolytic; the 400 m half stayed in Aerobic Power) · SAM V3 RULING 2: structure changed to DEPARTING EVERY 2:00 — ⚑ RATIO flag cleared, now genuinely in band</t>
+          <t>SPLIT from Aerobic Power's '200m/400m Repeats' (200 m ≈30 s is glycolytic; the 400 m half stayed in Aerobic Power) · SAM V3 RULING 2: DEPARTING EVERY 2:00 — ⚑ RATIO flag cleared, now genuinely in band</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -9170,7 +9044,7 @@
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>⚑ RATIO ≈2:1 vs band 1:2–1:5 (circuit format is work-heavy). ⚑ INFERRED numbers.</t>
+          <t>IN BAND. CLASSIFIED BY INTENSITY (Sam's V3-final law: intensity classifies, W:R is only a property). Sustained hard circuit intensity classifies it in Anaerobic; the work-heavy ratio is a property of the circuit format. ⚑ INFERRED numbers — the only mark left on this row.</t>
         </is>
       </c>
       <c r="J10" s="8" t="inlineStr">
@@ -9492,134 +9366,134 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>MAS 15:15 Blocks</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>MOVED from Anaerobic — 1:1 at 110% MAS is the framework's short-intermittent aerobic-power family (its own 30:15 session), not glycolytic 1:2–1:5 + MERGED — folds in ⚑ 'Broken 15s Ladder'</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>15 s hard</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>15 s easy</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>8 rounds × 2–3 blocks, 2 min between blocks</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>110% MAS (15 s work per masIntensityForWorkSeconds, src/utils/masCopy.ts)</t>
         </is>
       </c>
-      <c r="G5" s="8" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="H5" s="8" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>≈12–19 min (hard work 4–6 min)</t>
         </is>
       </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>W:R IN BAND. ⚑ BAND: 15 s effort is below the 1–5 min column — the framework's own 30:15 session sets the short-intermittent precedent.</t>
-        </is>
-      </c>
-      <c r="J5" s="8" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>IN BAND. CLASSIFIED BY INTENSITY (Sam's V3-final law: intensity classifies, W:R is only a property). 110% MAS is aerobic-power intensity, so the row classifies here; the 15 s effort length (below the 1–5 min column) is a property. The framework's own 30:15 session is the precedent.</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>15 seconds is short enough to go hard — actually go hard.</t>
         </is>
       </c>
-      <c r="K5" s="8" t="inlineStr">
+      <c r="K5" s="5" t="inlineStr">
         <is>
           <t>time</t>
         </is>
       </c>
-      <c r="L5" s="8" t="inlineStr">
+      <c r="L5" s="5" t="inlineStr">
         <is>
           <t>All 5 modalities — time-based, well inside the cap.</t>
         </is>
       </c>
-      <c r="M5" s="8" t="inlineStr">
+      <c r="M5" s="5" t="inlineStr">
         <is>
           <t>Bible L1271 / L1260 / L559; census 'MAS 15:15 Blocks'; framework's short-intermittent 100–110% MAS intensity line</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>30:30 Hard Intermittent</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>MOVED from Anaerobic (was ⚑ '30:30 Short Circuit') — 1:1 with repeatable-hard intent is aerobic-power-shaped, not glycolytic</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>30 s hard</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>30 s easy</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>8–10 rounds</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>100–110% MAS — hard and repeatable</t>
         </is>
       </c>
-      <c r="G6" s="8" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="H6" s="8" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>8–10 min (hard work 4–5 min)</t>
         </is>
       </c>
-      <c r="I6" s="8" t="inlineStr">
-        <is>
-          <t>W:R IN BAND. ⚑ BAND: 30 s effort below the 1–5 min column (same 30:15 precedent as above).</t>
-        </is>
-      </c>
-      <c r="J6" s="8" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>IN BAND. CLASSIFIED BY INTENSITY (Sam's V3-final law: intensity classifies, W:R is only a property). 100–110% MAS is aerobic-power intensity; the 30 s effort length is a property (same 30:15 precedent as above).</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>Hard, but it has to be repeatable for 8–10 rounds — not a sprint.</t>
         </is>
       </c>
-      <c r="K6" s="8" t="inlineStr">
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>time</t>
         </is>
       </c>
-      <c r="L6" s="8" t="inlineStr">
+      <c r="L6" s="5" t="inlineStr">
         <is>
           <t>All 5 modalities. Distinguish clearly from Aerobic Capacity's controlled 30:30, which is a tempo template.</t>
         </is>
       </c>
-      <c r="M6" s="8" t="inlineStr">
+      <c r="M6" s="5" t="inlineStr">
         <is>
           <t>Bible L1341 read as the harder variant; framework's 100–110% MAS short-intermittent line</t>
         </is>
@@ -9760,69 +9634,69 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>400 m Repeats</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>MOVED (GRIND DISSOLVED) + MERGED with the 400 m half of '200m/400m Repeats' — the state sheet's cross-listing is now resolved: 400 m (≈75–80 s) is aerobic-power length, 200 m went to Anaerobic</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>MOVED (GRIND DISSOLVED) + MERGED with the 400 m half of '200m/400m Repeats' · SAM V3-FINAL RULING 2: structure changed to DEPARTING EVERY 3:00 — ⚑ RATIO flag cleared</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>75–80 s (400 m)</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>2 min</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="inlineStr">
-        <is>
-          <t>4–6 reps</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Remainder of a 3:00 departure cycle (≈100–105 s)</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>4–6 reps, departing every 3:00</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>Hard, controlled — should genuinely hurt by rep 3</t>
         </is>
       </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>1:1.6</t>
-        </is>
-      </c>
-      <c r="H9" s="8" t="inlineStr">
-        <is>
-          <t>≈13–20 min</t>
-        </is>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>⚑ RATIO 1:1.6 vs band 1:1–2:1 (rest exceeds work). Rest ≈75–80 s would put it in band — Sam's call, not silently changed.</t>
-        </is>
-      </c>
-      <c r="J9" s="8" t="inlineStr">
-        <is>
-          <t>Hold your pace — it should genuinely hurt by rep 3, and rep 6 should still look like rep 1.</t>
-        </is>
-      </c>
-      <c r="K9" s="8" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>≈1:1.3 (1:1 for an athlete running ≈90 s)</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>12–18 min</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>IN BAND. CLASSIFIED BY INTENSITY (Sam's V3-final law: intensity classifies, W:R is only a property). Aerobic-power intensity classifies it here, and Sam's V3-final ruling 2 (departing every 3:00) brings the ratio to ~1:1-ish as well. Ratio flag cleared.</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>Hold your pace — it should genuinely hurt by rep 3, and rep 6 should still look like rep 1. The clock is the rest: you leave every 3:00.</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
         <is>
           <t>distance (400 m ≈ 75–80 s)</t>
         </is>
       </c>
-      <c r="L9" s="8" t="inlineStr">
-        <is>
-          <t>Run/Ski/Row: same nominal distance. Bike: 800 m. Air Bike: time via 250 m ≈ 1 min —&gt; ≈96 s.</t>
-        </is>
-      </c>
-      <c r="M9" s="8" t="inlineStr">
-        <is>
-          <t>Bible L1261 / L566; census '200m/400m Repeat Runs'</t>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>Run/Ski/Row: same nominal distance. Bike: 800 m. Air Bike: time via 250 m ≈ 1 min (≈96 s).</t>
+        </is>
+      </c>
+      <c r="M9" s="5" t="inlineStr">
+        <is>
+          <t>Bible L1261 / L566; census '200m/400m Repeat Runs'; re-structured by Sam's V3-final ruling 2</t>
         </is>
       </c>
     </row>
@@ -9869,7 +9743,7 @@
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>W:R IN BAND. ⚑ BAND: 40 s effort below the 1–5 min column (30:15 precedent). ⚑ INFERRED per-minute split.</t>
+          <t>IN BAND. CLASSIFIED BY INTENSITY (Sam's V3-final law: intensity classifies, W:R is only a property). Hard aerobic intensity classifies it here; the 40 s effort length is a property (30:15 precedent). ⚑ INFERRED per-minute split — the only mark left on this row.</t>
         </is>
       </c>
       <c r="J10" s="8" t="inlineStr">
@@ -10392,268 +10266,268 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Extensive Tempo (100 m repeats)</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>SCHEMA-FILLED + MERGED — folds in ⚑ 'Footy-Style Run-Throughs' (controlled run-throughs are this stimulus); dosed to the framework's session 3</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>≈16 s per 100 m</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>30 s walk between reps; 2–3 min between sets</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>2 sets × 8 reps</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>65–75% — game-speed rhythm, same pace every rep</t>
         </is>
       </c>
-      <c r="G8" s="8" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>≈1:2</t>
         </is>
       </c>
-      <c r="H8" s="8" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>≈15 min</t>
         </is>
       </c>
-      <c r="I8" s="8" t="inlineStr">
-        <is>
-          <t>⚑ RATIO ≈1:2 vs band 3:1–continuous — the whole tempo-interval family (30:30, 1:1, 2:1) sits outside the aerobic-capacity band. One systemic question, see Open Q3. LABEL CORRECTED to ~1:2 by Sam's V3 ruling 3 (the framework's '~2:1' was a labelling error) — the SESSION IS UNCHANGED. The surviving flag is the band question in Open Q3, not the label.</t>
-        </is>
-      </c>
-      <c r="J8" s="8" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>CLASSIFIED BY INTENSITY (Sam's V3-final law: intensity classifies, W:R is only a property). Controlled tempo intensity (65–80% MAS) puts this in Aerobic Capacity; its aerobic-power-shaped W:R is a property of the session, not a misfiling. Sam V3-final ruling 1 — ratio flag cleared. Ratio label corrected to ~1:2 by V3 ruling 3 (the framework's '~2:1' was a labelling error); the session is unchanged.</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>Same pace every rep — that's the actual test here. Think game-speed rhythm, not a track session.</t>
         </is>
       </c>
-      <c r="K8" s="8" t="inlineStr">
+      <c r="K8" s="5" t="inlineStr">
         <is>
           <t>distance (100 m @65–75% ≈ 16 s)</t>
         </is>
       </c>
-      <c r="L8" s="8" t="inlineStr">
+      <c r="L8" s="5" t="inlineStr">
         <is>
           <t>Run/Ski/Row: same nominal distance. Bike: 200 m. Air Bike: time via 250 m ≈ 1 min (≈24 s).</t>
         </is>
       </c>
-      <c r="M8" s="8" t="inlineStr">
+      <c r="M8" s="5" t="inlineStr">
         <is>
           <t>Framework, Aerobic capacity session 3 ('Extensive tempo — 2×8×100 m @65–75%, walk 30 s, 2–3 min between sets'), ratio label corrected per Sam V3 ruling 3; Bible L1223 / L1224</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>2 min On / 1 min Easy</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>MERGED — folds in ⚑ 'Assault Bike / Air Bike Tempo Intervals' (machine rendering of this exact structure; its 30:30 alternative folds into the 30:30 row below)</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>2 min</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>1 min easy</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>6–8 rounds</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>70–80% MAS — builds, doesn't fully recover</t>
         </is>
       </c>
-      <c r="G9" s="8" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
-      <c r="H9" s="8" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>18–24 min</t>
         </is>
       </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>⚑ RATIO 2:1 vs band 3:1–continuous — the whole tempo-interval family (30:30, 1:1, 2:1) sits outside the aerobic-capacity band. One systemic question, see Open Q3.</t>
-        </is>
-      </c>
-      <c r="J9" s="8" t="inlineStr">
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>CLASSIFIED BY INTENSITY (Sam's V3-final law: intensity classifies, W:R is only a property). Controlled tempo intensity (65–80% MAS) puts this in Aerobic Capacity; its aerobic-power-shaped W:R is a property of the session, not a misfiling. Sam V3-final ruling 1 — ratio flag cleared.</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>The rest is short on purpose — this should build, not fully recover.</t>
         </is>
       </c>
-      <c r="K9" s="8" t="inlineStr">
+      <c r="K9" s="5" t="inlineStr">
         <is>
           <t>time</t>
         </is>
       </c>
-      <c r="L9" s="8" t="inlineStr">
+      <c r="L9" s="5" t="inlineStr">
         <is>
           <t>All 5 modalities (time-based, inside the cap).</t>
         </is>
       </c>
-      <c r="M9" s="8" t="inlineStr">
+      <c r="M9" s="5" t="inlineStr">
         <is>
           <t>Bible L1230 / L1226–1230; census 'Assault Bike Intervals' / 'Air Bike Sprints'</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>30:30 Controlled Tempo Blocks</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>kept (absorbs the 30:30 alternative from the merged Air Bike tempo row)</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>30 s on</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>30 s easy</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>10–16 rounds</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>65–80% MAS — controlled, NOT max</t>
         </is>
       </c>
-      <c r="G10" s="8" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="H10" s="8" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>10–16 min</t>
         </is>
       </c>
-      <c r="I10" s="8" t="inlineStr">
-        <is>
-          <t>⚑ RATIO 1:1 vs band 3:1–continuous — the whole tempo-interval family (30:30, 1:1, 2:1) sits outside the aerobic-capacity band. One systemic question, see Open Q3.</t>
-        </is>
-      </c>
-      <c r="J10" s="8" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>CLASSIFIED BY INTENSITY (Sam's V3-final law: intensity classifies, W:R is only a property). Controlled tempo intensity (65–80% MAS) puts this in Aerobic Capacity; its aerobic-power-shaped W:R is a property of the session, not a misfiling. Sam V3-final ruling 1 — ratio flag cleared.</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t>Controlled, not max — you should be able to hold a conversation in three words by the end, not one.</t>
         </is>
       </c>
-      <c r="K10" s="8" t="inlineStr">
+      <c r="K10" s="5" t="inlineStr">
         <is>
           <t>time</t>
         </is>
       </c>
-      <c r="L10" s="8" t="inlineStr">
+      <c r="L10" s="5" t="inlineStr">
         <is>
           <t>All 5 modalities. Distinguish clearly from Aerobic Power's 30:30 Hard Intermittent.</t>
         </is>
       </c>
-      <c r="M10" s="8" t="inlineStr">
+      <c r="M10" s="5" t="inlineStr">
         <is>
           <t>Bible L1228; census '30:30 Tempo Blocks'</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>1 min On / 1 min Easy Tempo</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>kept</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>1 min</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>1 min easy</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>8–12 rounds</t>
         </is>
       </c>
-      <c r="F11" s="8" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>65–80% MAS controlled tempo</t>
         </is>
       </c>
-      <c r="G11" s="8" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="H11" s="8" t="inlineStr">
+      <c r="H11" s="5" t="inlineStr">
         <is>
           <t>16–24 min</t>
         </is>
       </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>⚑ RATIO 1:1 vs band 3:1–continuous — the whole tempo-interval family (30:30, 1:1, 2:1) sits outside the aerobic-capacity band. One systemic question, see Open Q3.</t>
-        </is>
-      </c>
-      <c r="J11" s="8" t="inlineStr">
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>CLASSIFIED BY INTENSITY (Sam's V3-final law: intensity classifies, W:R is only a property). Controlled tempo intensity (65–80% MAS) puts this in Aerobic Capacity; its aerobic-power-shaped W:R is a property of the session, not a misfiling. Sam V3-final ruling 1 — ratio flag cleared.</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
         <is>
           <t>Same idea as the 30:30, longer rhythm — settle into it.</t>
         </is>
       </c>
-      <c r="K11" s="8" t="inlineStr">
+      <c r="K11" s="5" t="inlineStr">
         <is>
           <t>time</t>
         </is>
       </c>
-      <c r="L11" s="8" t="inlineStr">
+      <c r="L11" s="5" t="inlineStr">
         <is>
           <t>All 5 modalities (time-based, inside the cap).</t>
         </is>
       </c>
-      <c r="M11" s="8" t="inlineStr">
+      <c r="M11" s="5" t="inlineStr">
         <is>
           <t>Bible L1229; census 'Tempo Intervals (1min on / 1min easy)'</t>
         </is>

</xml_diff>